<commit_message>
Restructure month sheets to 5-week internship months and fill 1st month
- Rebuilt sheet structure: each month sheet now spans 5 full weeks of
  internship from the start date (no calendar-month splits, no week-
  number overlap across sheets). 5 sheets used (1ος-5ος), 6ος cleared.
- Filled W1-W5 daily entries and weekly notes in 1ος (16/3 - 17/4),
  monthly trainee report and supervisor monthly report.
- Filled W6 daily entries and weekly notes in 2ος (20-24/4).
- Rewired the running-totals chain so extra!L13 points to 5ος!L69.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Βιβλίο Πρακτικής - Μελέτση.xlsx
+++ b/docs/Βιβλίο Πρακτικής - Μελέτση.xlsx
@@ -922,7 +922,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="204">
+  <cellXfs count="203">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1436,7 +1436,7 @@
     <xf numFmtId="167" fontId="15" fillId="7" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="15" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="7" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1547,9 +1547,6 @@
     </xf>
     <xf numFmtId="169" fontId="3" fillId="2" borderId="6" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2474,7 +2471,7 @@
           <t>Ημ/νία Λήξης βάσει Σύμβασης:</t>
         </is>
       </c>
-      <c r="C24" s="203" t="n">
+      <c r="C24" s="157" t="n">
         <v>46265</v>
       </c>
       <c r="D24" s="56">
@@ -3353,7 +3350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N78"/>
+  <dimension ref="B1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -3444,8 +3441,14 @@
         <f>D3</f>
         <v/>
       </c>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="26" t="n"/>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Καλωσόρισμα στα γραφεία της PwC στην Αθήνα. Παροχή εξοπλισμού.</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F7" s="166" t="n"/>
       <c r="G7" s="167" t="n"/>
       <c r="H7" s="167" t="n"/>
@@ -3460,8 +3463,14 @@
         <f>B7+1</f>
         <v/>
       </c>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="26" t="n"/>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Δεύτερη μέρα στα γραφεία της PwC. Συνάντηση με την ομάδα, Manager και Senior Software Engineer.</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F8" s="168" t="n"/>
       <c r="G8" s="169" t="n"/>
       <c r="H8" s="169" t="n"/>
@@ -3476,23 +3485,17 @@
         <f>B8+1</f>
         <v/>
       </c>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="26" t="n"/>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Remote εργασία. Πέρασα τις αποδείξεις ως εξοδολόγια με τη βοήθεια του senior — μου εξήγησε πώς θα δουλεύω και με ποιες εφαρμογές.</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F9" s="170" t="inlineStr">
         <is>
-          <t>- Ο ασκούμενος γράφει ΜΟΝΟ σε πράσινα κελιά.
-- Οι εβδομάδες ξεκινούν πάντα Δευτέρα και λήγουν Παρασκευή.
-   Αυτό προκύπτει αυτόματα εφόσον το κελί D3 (όταν είναι πράσινο)
-   συμπληρωθεί σωστά.
-- Κάθε μήνας έχει χώρο 5 εβδομάδων. Χρησιμοποιήστε ΜΟΝΟ όσες
-   χρειάζονται για να ολοκληρωθεί ο μήνας. Μετά αλλάξτε φύλλο.
-- Σε φύλλο δεδομένου μήνα, χρησιμοποήστε ΜΟΝΟ τις μέρες αυτού
-   του μήνα. Τυχόν μέρες άλλων μηνών (στην αρχή ή στο τέλος του
-   φύλλου) θα πρέπει να αφήνονται κενές.
-- Εβδομάδα που μοιράζεται σε 2 μήνες, θα πρέπει να έχει ίδιο
-   αύξοντα αριθμό. Αν δεν έχει, τότε συμπληρώσατε λάθος το D3.
-- Σε ημέρες που δεν εργαστήκατε να αναγράφετε τον λόγο (π.χ. Αργία 
-   Εθνική Εορτή, κτλ). και να αφήνετε ΚΕΝΟ το κελί ωρών εργασίας.</t>
+          <t>Είχα ένα θερμό καλωσόρισμα από την ομάδα και την εταιρεία. Μου εξήγησαν αναλυτικά τι πρέπει να κάνω και με βοήθησαν να προσαρμοστώ. Έκανα μια αρχή σε βάση δεδομένων — εκπαιδευτικό, όχι πραγματικό έργο.</t>
         </is>
       </c>
       <c r="G9" s="171" t="n"/>
@@ -3508,8 +3511,14 @@
         <f>B9+1</f>
         <v/>
       </c>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="26" t="n"/>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>2 υποχρεωτικά online courses σχετικά με την εταιρεία και τις αρμοδιότητές μου (εκπαίδευση κανόνων και προσαρμογής). Εβδομαδιαίο meeting με την ομάδα του .NET.</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F10" s="173" t="n"/>
       <c r="M10" s="174" t="n"/>
     </row>
@@ -3518,8 +3527,14 @@
         <f>B10+1</f>
         <v/>
       </c>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="29" t="n"/>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Visual Studio Subscription. GitHub Enterprise Cloud — ticket form Hub. SQL courses και σχεδιασμός βάσης δεδομένων για εκπαιδευτικό έργο σχολείων Αττικής (μη πραγματικό έργο).</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>8</v>
+      </c>
       <c r="F11" s="175" t="n"/>
       <c r="G11" s="176" t="n"/>
       <c r="H11" s="176" t="n"/>
@@ -3644,8 +3659,14 @@
         <f>D17</f>
         <v/>
       </c>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="26" t="n"/>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Meeting με τον manager. Meeting με την ομάδα για απορίες. Συνέχεια της βάσης δεδομένων από την προηγούμενη εβδομάδα.</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F21" s="179" t="n"/>
       <c r="G21" s="167" t="n"/>
       <c r="H21" s="167" t="n"/>
@@ -3660,8 +3681,14 @@
         <f>B21+1</f>
         <v/>
       </c>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="26" t="n"/>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Online eLearn με το HC. Cloud Platforms Interns sync — αναφορά εργασιών προηγούμενων ημερών. Διόρθωση βάσης δεδομένων μετά από συζήτηση με senior και manager.</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F22" s="168" t="n"/>
       <c r="G22" s="169" t="n"/>
       <c r="H22" s="169" t="n"/>
@@ -3676,11 +3703,16 @@
         <f>B22+1</f>
         <v/>
       </c>
-      <c r="C23" s="22" t="n"/>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>Αργία — 25η Μαρτίου (Εθνική Εορτή).</t>
+        </is>
+      </c>
       <c r="D23" s="26" t="n"/>
-      <c r="F23" s="180">
-        <f>F9</f>
-        <v/>
+      <c r="F23" s="180" t="inlineStr">
+        <is>
+          <t>Όλα εξελίσσονται ομαλά και ευχάριστα και συνεχίζω ό,τι μου είχε ανατεθεί.</t>
+        </is>
       </c>
       <c r="G23" s="171" t="n"/>
       <c r="H23" s="171" t="n"/>
@@ -3695,8 +3727,14 @@
         <f>B23+1</f>
         <v/>
       </c>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="26" t="n"/>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>Meeting team .NET. Τελική διόρθωση και ολοκλήρωση του διαγράμματος ERD. Έναρξη δημιουργίας πινάκων σε MySQL / SQL Studio.</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F24" s="173" t="n"/>
       <c r="M24" s="174" t="n"/>
     </row>
@@ -3705,8 +3743,14 @@
         <f>B24+1</f>
         <v/>
       </c>
-      <c r="C25" s="23" t="n"/>
-      <c r="D25" s="29" t="n"/>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Meeting team sync. Συνέχεια SQL και δημιουργία tickets στο IT για πρόσβαση σε εφαρμογές που θα χρειαστούν αργότερα.</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>8</v>
+      </c>
       <c r="F25" s="175" t="n"/>
       <c r="G25" s="176" t="n"/>
       <c r="H25" s="176" t="n"/>
@@ -3748,27 +3792,73 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="74" t="n"/>
-    </row>
-    <row r="30"/>
+      <c r="B29" s="74" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
+        </is>
+      </c>
+    </row>
     <row r="31" ht="18.75" customHeight="1">
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="178" t="n"/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΑ</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>από Δευτέρα:</t>
+        </is>
+      </c>
+      <c r="D31" s="32">
+        <f>D17+7</f>
+        <v/>
+      </c>
+      <c r="E31" s="178">
+        <f>D31</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="18.75" customHeight="1">
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="31" t="n"/>
-      <c r="E32" s="178" t="n"/>
-    </row>
-    <row r="33"/>
+      <c r="B32" s="12">
+        <f>B18+1</f>
+        <v/>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>έως Παρασκευή:</t>
+        </is>
+      </c>
+      <c r="D32" s="31">
+        <f>D31+4</f>
+        <v/>
+      </c>
+      <c r="E32" s="178">
+        <f>D32</f>
+        <v/>
+      </c>
+    </row>
     <row r="34" ht="31.5" customHeight="1">
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="13" t="n"/>
-      <c r="F34" s="77" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>ΗΜΕΡΑ</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
+ ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>ΩΡΕΣ</t>
+        </is>
+      </c>
+      <c r="F34" s="77" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
+        </is>
+      </c>
       <c r="G34" s="164" t="n"/>
       <c r="H34" s="164" t="n"/>
       <c r="I34" s="164" t="n"/>
@@ -3778,9 +3868,18 @@
       <c r="M34" s="165" t="n"/>
     </row>
     <row r="35" ht="76.5" customHeight="1">
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="26" t="n"/>
+      <c r="B35" s="24">
+        <f>D31</f>
+        <v/>
+      </c>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>Meeting team. Meeting με τον manager. Συνέχεια SQL — ολοκλήρωση πινάκων και αποστολή στον senior για διόρθωση. Παρακολούθηση courses για React.</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F35" s="179" t="n"/>
       <c r="G35" s="167" t="n"/>
       <c r="H35" s="167" t="n"/>
@@ -3791,9 +3890,18 @@
       <c r="M35" s="149" t="n"/>
     </row>
     <row r="36" ht="76.5" customHeight="1">
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="25" t="n"/>
-      <c r="D36" s="26" t="n"/>
+      <c r="B36" s="24">
+        <f>B35+1</f>
+        <v/>
+      </c>
+      <c r="C36" s="25" t="inlineStr">
+        <is>
+          <t>Internship program meeting. Online courses από Udemy (React, frontend &amp; backend) — υπόδειξη του manager.</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F36" s="168" t="n"/>
       <c r="G36" s="169" t="n"/>
       <c r="H36" s="169" t="n"/>
@@ -3804,10 +3912,23 @@
       <c r="M36" s="153" t="n"/>
     </row>
     <row r="37" ht="76.5" customHeight="1">
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="25" t="n"/>
-      <c r="D37" s="26" t="n"/>
-      <c r="F37" s="180" t="n"/>
+      <c r="B37" s="24">
+        <f>B36+1</f>
+        <v/>
+      </c>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team. Συνέχεια SQL: διόρθωση πινάκων μετά από παρατηρήσεις του senior. Ολοκλήρωση Database Assessment Part 1. Έναρξη Part 2 (25 queries σε Sakila DB) — κατέβασα τη βάση, την έτρεξα με τις οδηγίες και άρχισα να δημιουργώ τα queries.</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F37" s="180" t="inlineStr">
+        <is>
+          <t>Επικεντρώθηκα στην Database Assessment ώστε να την ολοκληρώσω. Part 1: ERD διάγραμμα και δημιουργία πινάκων σε MySQL. Part 2: Sakila database — απάντηση σε 25 queries.</t>
+        </is>
+      </c>
       <c r="G37" s="171" t="n"/>
       <c r="H37" s="171" t="n"/>
       <c r="I37" s="171" t="n"/>
@@ -3817,16 +3938,34 @@
       <c r="M37" s="172" t="n"/>
     </row>
     <row r="38" ht="76.5" customHeight="1">
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="26" t="n"/>
+      <c r="B38" s="24">
+        <f>B37+1</f>
+        <v/>
+      </c>
+      <c r="C38" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team .NET. Συνέχεια του Part 2 της Database Assessment. Διόρθωση Part 1 μετά τις παρατηρήσεις του senior.</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F38" s="173" t="n"/>
       <c r="M38" s="174" t="n"/>
     </row>
     <row r="39" ht="76.5" customHeight="1">
-      <c r="B39" s="27" t="n"/>
-      <c r="C39" s="28" t="n"/>
-      <c r="D39" s="29" t="n"/>
+      <c r="B39" s="27">
+        <f>B38+1</f>
+        <v/>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>Meeting with team. Συνέχεια Database Assessment Part 2. 2-ωρο ενημερωτικό meeting call με την εταιρεία.</t>
+        </is>
+      </c>
+      <c r="D39" s="29" t="n">
+        <v>8</v>
+      </c>
       <c r="F39" s="175" t="n"/>
       <c r="G39" s="176" t="n"/>
       <c r="H39" s="176" t="n"/>
@@ -3837,38 +3976,104 @@
       <c r="M39" s="177" t="n"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="16" t="n"/>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
+        </is>
+      </c>
+      <c r="D40" s="16">
+        <f>SUM(D35:D39)</f>
+        <v/>
+      </c>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="16" t="n"/>
-      <c r="K41" s="17" t="n"/>
-      <c r="L41" s="18" t="n"/>
-    </row>
-    <row r="42"/>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>Ημέρες Εργασίας Εβδομάδας:</t>
+        </is>
+      </c>
+      <c r="D41" s="16">
+        <f>COUNTA(D35:D39)</f>
+        <v/>
+      </c>
+      <c r="K41" s="17" t="inlineStr">
+        <is>
+          <t>Σύνολο Εργάσιμων Ημερών:</t>
+        </is>
+      </c>
+      <c r="L41" s="18">
+        <f>D41+L27</f>
+        <v/>
+      </c>
+    </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="B43" s="74" t="n"/>
-    </row>
-    <row r="44"/>
+      <c r="B43" s="74" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="18.75" customHeight="1">
-      <c r="B45" s="10" t="n"/>
-      <c r="C45" s="11" t="n"/>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="178" t="n"/>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΑ</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>από Δευτέρα:</t>
+        </is>
+      </c>
+      <c r="D45" s="32">
+        <f>D31+7</f>
+        <v/>
+      </c>
+      <c r="E45" s="178">
+        <f>D45</f>
+        <v/>
+      </c>
     </row>
     <row r="46" ht="18.75" customHeight="1">
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="31" t="n"/>
-      <c r="E46" s="178" t="n"/>
-    </row>
-    <row r="47"/>
+      <c r="B46" s="12">
+        <f>B32+1</f>
+        <v/>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>έως Παρασκευή:</t>
+        </is>
+      </c>
+      <c r="D46" s="31">
+        <f>D45+4</f>
+        <v/>
+      </c>
+      <c r="E46" s="178">
+        <f>D46</f>
+        <v/>
+      </c>
+    </row>
     <row r="48" ht="31.5" customHeight="1">
-      <c r="B48" s="13" t="n"/>
-      <c r="C48" s="14" t="n"/>
-      <c r="D48" s="13" t="n"/>
-      <c r="F48" s="77" t="n"/>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>ΗΜΕΡΑ</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
+ ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>ΩΡΕΣ</t>
+        </is>
+      </c>
+      <c r="F48" s="77" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
+        </is>
+      </c>
       <c r="G48" s="164" t="n"/>
       <c r="H48" s="164" t="n"/>
       <c r="I48" s="164" t="n"/>
@@ -3878,9 +4083,18 @@
       <c r="M48" s="165" t="n"/>
     </row>
     <row r="49" ht="76.5" customHeight="1">
-      <c r="B49" s="24" t="n"/>
-      <c r="C49" s="25" t="n"/>
-      <c r="D49" s="26" t="n"/>
+      <c r="B49" s="24">
+        <f>D45</f>
+        <v/>
+      </c>
+      <c r="C49" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team. Παράδοση Part 2 της Database Assessment στον senior για παρατηρήσεις. React courses.</t>
+        </is>
+      </c>
+      <c r="D49" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F49" s="179" t="n"/>
       <c r="G49" s="167" t="n"/>
       <c r="H49" s="167" t="n"/>
@@ -3891,9 +4105,18 @@
       <c r="M49" s="149" t="n"/>
     </row>
     <row r="50" ht="76.5" customHeight="1">
-      <c r="B50" s="24" t="n"/>
-      <c r="C50" s="25" t="n"/>
-      <c r="D50" s="26" t="n"/>
+      <c r="B50" s="24">
+        <f>B49+1</f>
+        <v/>
+      </c>
+      <c r="C50" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with manager. Cloud platform internship. Διορθώσεις στο Part 2 → ολοκλήρωση της Database Assessment.</t>
+        </is>
+      </c>
+      <c r="D50" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F50" s="168" t="n"/>
       <c r="G50" s="169" t="n"/>
       <c r="H50" s="169" t="n"/>
@@ -3904,10 +4127,23 @@
       <c r="M50" s="153" t="n"/>
     </row>
     <row r="51" ht="76.5" customHeight="1">
-      <c r="B51" s="24" t="n"/>
-      <c r="C51" s="25" t="n"/>
-      <c r="D51" s="26" t="n"/>
-      <c r="F51" s="180" t="n"/>
+      <c r="B51" s="24">
+        <f>B50+1</f>
+        <v/>
+      </c>
+      <c r="C51" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team &amp; .NET. Παρακολούθηση υποχρεωτικών AI courses (1/3).</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F51" s="180" t="inlineStr">
+        <is>
+          <t>Ολοκλήρωση της Database Assessment. Παρακολούθηση courses (AI &amp; React).</t>
+        </is>
+      </c>
       <c r="G51" s="171" t="n"/>
       <c r="H51" s="171" t="n"/>
       <c r="I51" s="171" t="n"/>
@@ -3917,15 +4153,29 @@
       <c r="M51" s="172" t="n"/>
     </row>
     <row r="52" ht="76.5" customHeight="1">
-      <c r="B52" s="24" t="n"/>
-      <c r="C52" s="25" t="n"/>
+      <c r="B52" s="24">
+        <f>B51+1</f>
+        <v/>
+      </c>
+      <c r="C52" s="25" t="inlineStr">
+        <is>
+          <t>Εταιρεία κλειστή λόγω Πάσχα (Μεγάλη Πέμπτη).</t>
+        </is>
+      </c>
       <c r="D52" s="26" t="n"/>
       <c r="F52" s="173" t="n"/>
       <c r="M52" s="174" t="n"/>
     </row>
     <row r="53" ht="76.5" customHeight="1">
-      <c r="B53" s="27" t="n"/>
-      <c r="C53" s="28" t="n"/>
+      <c r="B53" s="27">
+        <f>B52+1</f>
+        <v/>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>Αργία — Μεγάλη Παρασκευή.</t>
+        </is>
+      </c>
       <c r="D53" s="29" t="n"/>
       <c r="F53" s="175" t="n"/>
       <c r="G53" s="176" t="n"/>
@@ -3937,38 +4187,104 @@
       <c r="M53" s="177" t="n"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
-      <c r="C54" s="15" t="n"/>
-      <c r="D54" s="16" t="n"/>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
+        </is>
+      </c>
+      <c r="D54" s="16">
+        <f>SUM(D49:D53)</f>
+        <v/>
+      </c>
     </row>
     <row r="55" ht="19.5" customHeight="1">
-      <c r="C55" s="15" t="n"/>
-      <c r="D55" s="16" t="n"/>
-      <c r="K55" s="17" t="n"/>
-      <c r="L55" s="18" t="n"/>
-    </row>
-    <row r="56"/>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Ημέρες Εργασίας Εβδομάδας:</t>
+        </is>
+      </c>
+      <c r="D55" s="16">
+        <f>COUNTA(D49:D53)</f>
+        <v/>
+      </c>
+      <c r="K55" s="17" t="inlineStr">
+        <is>
+          <t>Σύνολο Εργάσιμων Ημερών:</t>
+        </is>
+      </c>
+      <c r="L55" s="18">
+        <f>D55+L41</f>
+        <v/>
+      </c>
+    </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="74" t="n"/>
-    </row>
-    <row r="58"/>
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
+        </is>
+      </c>
+    </row>
     <row r="59" ht="18.75" customHeight="1">
-      <c r="B59" s="10" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="32" t="n"/>
-      <c r="E59" s="178" t="n"/>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΑ</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>από Δευτέρα:</t>
+        </is>
+      </c>
+      <c r="D59" s="32">
+        <f>D45+7</f>
+        <v/>
+      </c>
+      <c r="E59" s="178">
+        <f>D59</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="18.75" customHeight="1">
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="11" t="n"/>
-      <c r="D60" s="31" t="n"/>
-      <c r="E60" s="178" t="n"/>
-    </row>
-    <row r="61"/>
+      <c r="B60" s="12">
+        <f>B46+1</f>
+        <v/>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>έως Παρασκευή:</t>
+        </is>
+      </c>
+      <c r="D60" s="31">
+        <f>D59+4</f>
+        <v/>
+      </c>
+      <c r="E60" s="178">
+        <f>D60</f>
+        <v/>
+      </c>
+    </row>
     <row r="62" ht="31.5" customHeight="1">
-      <c r="B62" s="13" t="n"/>
-      <c r="C62" s="14" t="n"/>
-      <c r="D62" s="13" t="n"/>
-      <c r="F62" s="77" t="n"/>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>ΗΜΕΡΑ</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
+ ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>ΩΡΕΣ</t>
+        </is>
+      </c>
+      <c r="F62" s="77" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
+        </is>
+      </c>
       <c r="G62" s="164" t="n"/>
       <c r="H62" s="164" t="n"/>
       <c r="I62" s="164" t="n"/>
@@ -3978,8 +4294,15 @@
       <c r="M62" s="165" t="n"/>
     </row>
     <row r="63" ht="76.5" customHeight="1">
-      <c r="B63" s="24" t="n"/>
-      <c r="C63" s="25" t="n"/>
+      <c r="B63" s="24">
+        <f>D59</f>
+        <v/>
+      </c>
+      <c r="C63" s="25" t="inlineStr">
+        <is>
+          <t>Αργία — Δευτέρα του Πάσχα.</t>
+        </is>
+      </c>
       <c r="D63" s="26" t="n"/>
       <c r="F63" s="179" t="n"/>
       <c r="G63" s="167" t="n"/>
@@ -3991,8 +4314,15 @@
       <c r="M63" s="149" t="n"/>
     </row>
     <row r="64" ht="76.5" customHeight="1">
-      <c r="B64" s="24" t="n"/>
-      <c r="C64" s="25" t="n"/>
+      <c r="B64" s="24">
+        <f>B63+1</f>
+        <v/>
+      </c>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>Εταιρεία κλειστή λόγω Πάσχα.</t>
+        </is>
+      </c>
       <c r="D64" s="26" t="n"/>
       <c r="F64" s="168" t="n"/>
       <c r="G64" s="169" t="n"/>
@@ -4004,10 +4334,23 @@
       <c r="M64" s="153" t="n"/>
     </row>
     <row r="65" ht="76.5" customHeight="1">
-      <c r="B65" s="24" t="n"/>
-      <c r="C65" s="25" t="n"/>
-      <c r="D65" s="26" t="n"/>
-      <c r="F65" s="180" t="n"/>
+      <c r="B65" s="24">
+        <f>B64+1</f>
+        <v/>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team. Παρακολούθηση των υπολοίπων AI courses (3/3) και συνέχεια των React courses στο Udemy.</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F65" s="180" t="inlineStr">
+        <is>
+          <t>Ήταν μια εβδομάδα με αρκετό διάβασμα και πολλές πληροφορίες για AI και React.</t>
+        </is>
+      </c>
       <c r="G65" s="171" t="n"/>
       <c r="H65" s="171" t="n"/>
       <c r="I65" s="171" t="n"/>
@@ -4017,16 +4360,34 @@
       <c r="M65" s="172" t="n"/>
     </row>
     <row r="66" ht="76.5" customHeight="1">
-      <c r="B66" s="24" t="n"/>
-      <c r="C66" s="25" t="n"/>
-      <c r="D66" s="26" t="n"/>
+      <c r="B66" s="24">
+        <f>B65+1</f>
+        <v/>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>Meeting with team &amp; .NET. Παρακολούθηση courses for React.</t>
+        </is>
+      </c>
+      <c r="D66" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F66" s="173" t="n"/>
       <c r="M66" s="174" t="n"/>
     </row>
     <row r="67" ht="76.5" customHeight="1">
-      <c r="B67" s="27" t="n"/>
-      <c r="C67" s="28" t="n"/>
-      <c r="D67" s="29" t="n"/>
+      <c r="B67" s="27">
+        <f>B66+1</f>
+        <v/>
+      </c>
+      <c r="C67" s="28" t="inlineStr">
+        <is>
+          <t>Meeting with team. Παρακολούθηση courses for React.</t>
+        </is>
+      </c>
+      <c r="D67" s="29" t="n">
+        <v>8</v>
+      </c>
       <c r="F67" s="175" t="n"/>
       <c r="G67" s="176" t="n"/>
       <c r="H67" s="176" t="n"/>
@@ -4037,14 +4398,35 @@
       <c r="M67" s="177" t="n"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="C68" s="15" t="n"/>
-      <c r="D68" s="16" t="n"/>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
+        </is>
+      </c>
+      <c r="D68" s="16">
+        <f>SUM(D63:D67)</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="K69" s="17" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Ημέρες Εργασίας Εβδομάδας:</t>
+        </is>
+      </c>
+      <c r="D69" s="16">
+        <f>COUNTA(D63:D67)</f>
+        <v/>
+      </c>
+      <c r="K69" s="17" t="inlineStr">
+        <is>
+          <t>Σύνολο Εργάσιμων Ημερών:</t>
+        </is>
+      </c>
+      <c r="L69" s="18">
+        <f>D69+L55</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="16.5" customHeight="1">
       <c r="B73" s="181" t="inlineStr">
@@ -4056,7 +4438,11 @@
       <c r="D73" s="165" t="n"/>
     </row>
     <row r="74" ht="150" customHeight="1">
-      <c r="B74" s="166" t="n"/>
+      <c r="B74" s="166" t="inlineStr">
+        <is>
+          <t>Είχα μια ομαλή και ευχάριστη προσαρμογή στην εταιρεία με πολλή καθοδήγηση και υποστήριξη από την ομάδα. Σε αυτόν τον μήνα ολοκλήρωσα το πρώτο training, που ήταν μια Database Assessment για σχολεία της Αττικής. Παρακολούθησα κάποια courses σχετικά με τη React (frontend &amp; backend) αλλά και κάποια courses για το AI.</t>
+        </is>
+      </c>
       <c r="C74" s="182" t="n"/>
       <c r="D74" s="183" t="n"/>
     </row>
@@ -4070,7 +4456,11 @@
       <c r="D77" s="165" t="n"/>
     </row>
     <row r="78" ht="150" customHeight="1">
-      <c r="B78" s="184" t="n"/>
+      <c r="B78" s="184" t="inlineStr">
+        <is>
+          <t>Η ασκούμενη Παρασκευή Μελέτση παρουσίασε εξαιρετική αρχική εικόνα κατά τον πρώτο μήνα της πρακτικής της. Επιδεικνύει έντονη όρεξη για μάθηση και διατηρεί σταθερά θετική και συνεργατική στάση απέναντι στους συναδέλφους της. Με αρκετά καλές τεχνικές βάσεις ενσωματώθηκε γρήγορα στο περιβάλλον εργασίας, και στο πρώτο της assessment (Database Assessment) η πρόοδός της υπήρξε ταχεία και υψηλής ποιότητας, αξιοποιώντας ουσιαστικά το feedback που της δόθηκε. Διακρίνεται για την ικανότητά της να διατηρεί οργανωμένο το προσωπικό της roadmap, λειτουργώντας ανεξάρτητα στις καθημερινές της εργασίες αλλά και ζητώντας στοχευμένη καθοδήγηση για τα επόμενα βήματα ώστε να παραμένει σταθερά στην επιθυμητή πορεία. Ο πρώτος μήνας ολοκληρώνεται με ιδιαίτερα θετικές προοπτικές για τη συνέχεια.</t>
+        </is>
+      </c>
       <c r="C78" s="182" t="n"/>
       <c r="D78" s="183" t="n"/>
     </row>
@@ -4134,7 +4524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N78"/>
+  <dimension ref="B1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -4164,7 +4554,7 @@
         </is>
       </c>
       <c r="D3" s="185" t="n">
-        <v>46111</v>
+        <v>46132</v>
       </c>
       <c r="E3" s="178">
         <f>D3</f>
@@ -4225,8 +4615,14 @@
         <f>D3</f>
         <v/>
       </c>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="26" t="n"/>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Course για τη React και τα API keys → ολοκλήρωση πρώτου course. Meeting with team and manager.</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F7" s="166" t="n"/>
       <c r="G7" s="167" t="n"/>
       <c r="H7" s="167" t="n"/>
@@ -4241,8 +4637,14 @@
         <f>B7+1</f>
         <v/>
       </c>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="26" t="n"/>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Meeting Cloud platform internship. Έναρξη Web Calculator training — εμφάνιση UI σε React και βασικές λειτουργίες (+, −, ×, ÷).</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F8" s="168" t="n"/>
       <c r="G8" s="169" t="n"/>
       <c r="H8" s="169" t="n"/>
@@ -4257,11 +4659,18 @@
         <f>B8+1</f>
         <v/>
       </c>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="26" t="n"/>
-      <c r="F9" s="180">
-        <f>'1ος'!F9:M11</f>
-        <v/>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Meeting with team. Course για τη React (για να συνεχίσω το calculator). Αλλαγές στον calculator και συνέχεια του training.</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="180" t="inlineStr">
+        <is>
+          <t>Ξεκίνησα το Web Calculator training μετά την ολοκλήρωση των courses στη React.</t>
+        </is>
       </c>
       <c r="G9" s="171" t="n"/>
       <c r="H9" s="171" t="n"/>
@@ -4276,8 +4685,14 @@
         <f>B9+1</f>
         <v/>
       </c>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="26" t="n"/>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Meeting with team. AI use case series — ενημερωτικό από την εταιρεία. Συνέχεια του calculator — προσθήκη ιστορικού πράξεων.</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="F10" s="173" t="n"/>
       <c r="M10" s="174" t="n"/>
     </row>
@@ -4286,8 +4701,14 @@
         <f>B10+1</f>
         <v/>
       </c>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="29" t="n"/>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Meeting with team. Συνέχεια στο calculator history με καλύτερες τεχνικές.</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>8</v>
+      </c>
       <c r="F11" s="175" t="n"/>
       <c r="G11" s="176" t="n"/>
       <c r="H11" s="176" t="n"/>
@@ -4324,7 +4745,7 @@
         </is>
       </c>
       <c r="L13" s="18">
-        <f>D13+'1ος'!L27</f>
+        <f>D13+'1ος'!L69</f>
         <v/>
       </c>
     </row>
@@ -4821,27 +5242,73 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="74" t="n"/>
-    </row>
-    <row r="58"/>
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
+        </is>
+      </c>
+    </row>
     <row r="59" ht="18.75" customHeight="1">
-      <c r="B59" s="10" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="32" t="n"/>
-      <c r="E59" s="163" t="n"/>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΑ</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>από Δευτέρα:</t>
+        </is>
+      </c>
+      <c r="D59" s="32">
+        <f>D45+7</f>
+        <v/>
+      </c>
+      <c r="E59" s="163">
+        <f>WEEKDAY(D59)</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="18.75" customHeight="1">
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="11" t="n"/>
-      <c r="D60" s="31" t="n"/>
-      <c r="E60" s="163" t="n"/>
-    </row>
-    <row r="61"/>
+      <c r="B60" s="12">
+        <f>B46+1</f>
+        <v/>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>έως Παρασκευή:</t>
+        </is>
+      </c>
+      <c r="D60" s="31">
+        <f>D59+4</f>
+        <v/>
+      </c>
+      <c r="E60" s="163">
+        <f>WEEKDAY(D60)</f>
+        <v/>
+      </c>
+    </row>
     <row r="62" ht="31.5" customHeight="1">
-      <c r="B62" s="13" t="n"/>
-      <c r="C62" s="14" t="n"/>
-      <c r="D62" s="13" t="n"/>
-      <c r="F62" s="77" t="n"/>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>ΗΜΕΡΑ</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
+ ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>ΩΡΕΣ</t>
+        </is>
+      </c>
+      <c r="F62" s="77" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
+        </is>
+      </c>
       <c r="G62" s="164" t="n"/>
       <c r="H62" s="164" t="n"/>
       <c r="I62" s="164" t="n"/>
@@ -4851,7 +5318,10 @@
       <c r="M62" s="165" t="n"/>
     </row>
     <row r="63" ht="76.5" customHeight="1">
-      <c r="B63" s="24" t="n"/>
+      <c r="B63" s="24">
+        <f>D59</f>
+        <v/>
+      </c>
       <c r="C63" s="25" t="n"/>
       <c r="D63" s="26" t="n"/>
       <c r="F63" s="179" t="n"/>
@@ -4864,7 +5334,10 @@
       <c r="M63" s="149" t="n"/>
     </row>
     <row r="64" ht="76.5" customHeight="1">
-      <c r="B64" s="24" t="n"/>
+      <c r="B64" s="24">
+        <f>B63+1</f>
+        <v/>
+      </c>
       <c r="C64" s="25" t="n"/>
       <c r="D64" s="26" t="n"/>
       <c r="F64" s="168" t="n"/>
@@ -4877,29 +5350,59 @@
       <c r="M64" s="153" t="n"/>
     </row>
     <row r="65" ht="76.5" customHeight="1">
-      <c r="B65" s="24" t="n"/>
+      <c r="B65" s="24">
+        <f>B64+1</f>
+        <v/>
+      </c>
       <c r="C65" s="25" t="n"/>
       <c r="D65" s="26" t="n"/>
     </row>
     <row r="66" ht="76.5" customHeight="1">
-      <c r="B66" s="24" t="n"/>
+      <c r="B66" s="24">
+        <f>B65+1</f>
+        <v/>
+      </c>
       <c r="C66" s="25" t="n"/>
       <c r="D66" s="26" t="n"/>
     </row>
     <row r="67" ht="76.5" customHeight="1">
-      <c r="B67" s="27" t="n"/>
+      <c r="B67" s="27">
+        <f>B66+1</f>
+        <v/>
+      </c>
       <c r="C67" s="28" t="n"/>
       <c r="D67" s="29" t="n"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="C68" s="15" t="n"/>
-      <c r="D68" s="16" t="n"/>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
+        </is>
+      </c>
+      <c r="D68" s="16">
+        <f>SUM(D63:D67)</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="K69" s="17" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Ημέρες Εργασίας Εβδομάδας:</t>
+        </is>
+      </c>
+      <c r="D69" s="16">
+        <f>COUNTA(D63:D67)</f>
+        <v/>
+      </c>
+      <c r="K69" s="17" t="inlineStr">
+        <is>
+          <t>Σύνολο Εργάσιμων Ημερών:</t>
+        </is>
+      </c>
+      <c r="L69" s="18">
+        <f>D69+L55</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="16.5" customHeight="1">
       <c r="B73" s="181" t="inlineStr">
@@ -5015,7 +5518,7 @@
         </is>
       </c>
       <c r="D3" s="185" t="n">
-        <v>46139</v>
+        <v>46167</v>
       </c>
       <c r="E3" s="163">
         <f>WEEKDAY(D3)</f>
@@ -5175,7 +5678,7 @@
         </is>
       </c>
       <c r="L13" s="18">
-        <f>D13+'2ος'!L55</f>
+        <f>D13+'2ος'!L69</f>
         <v/>
       </c>
     </row>
@@ -5918,7 +6421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N78"/>
+  <dimension ref="B1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -5948,7 +6451,7 @@
         </is>
       </c>
       <c r="D3" s="185" t="n">
-        <v>46174</v>
+        <v>46202</v>
       </c>
       <c r="E3" s="163">
         <f>WEEKDAY(D3)</f>
@@ -6605,27 +7108,73 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="74" t="n"/>
-    </row>
-    <row r="58"/>
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
+        </is>
+      </c>
+    </row>
     <row r="59" ht="18.75" customHeight="1">
-      <c r="B59" s="10" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="32" t="n"/>
-      <c r="E59" s="178" t="n"/>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΑ</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>από Δευτέρα:</t>
+        </is>
+      </c>
+      <c r="D59" s="32">
+        <f>D45+7</f>
+        <v/>
+      </c>
+      <c r="E59" s="178">
+        <f>D59</f>
+        <v/>
+      </c>
     </row>
     <row r="60" ht="18.75" customHeight="1">
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="11" t="n"/>
-      <c r="D60" s="31" t="n"/>
-      <c r="E60" s="178" t="n"/>
-    </row>
-    <row r="61"/>
+      <c r="B60" s="12">
+        <f>B46+1</f>
+        <v/>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>έως Παρασκευή:</t>
+        </is>
+      </c>
+      <c r="D60" s="31">
+        <f>D59+4</f>
+        <v/>
+      </c>
+      <c r="E60" s="178">
+        <f>D60</f>
+        <v/>
+      </c>
+    </row>
     <row r="62" ht="31.5" customHeight="1">
-      <c r="B62" s="13" t="n"/>
-      <c r="C62" s="14" t="n"/>
-      <c r="D62" s="13" t="n"/>
-      <c r="F62" s="77" t="n"/>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>ΗΜΕΡΑ</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
+ ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>ΩΡΕΣ</t>
+        </is>
+      </c>
+      <c r="F62" s="77" t="inlineStr">
+        <is>
+          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
+        </is>
+      </c>
       <c r="G62" s="164" t="n"/>
       <c r="H62" s="164" t="n"/>
       <c r="I62" s="164" t="n"/>
@@ -6635,7 +7184,10 @@
       <c r="M62" s="165" t="n"/>
     </row>
     <row r="63" ht="76.5" customHeight="1">
-      <c r="B63" s="24" t="n"/>
+      <c r="B63" s="24">
+        <f>D59</f>
+        <v/>
+      </c>
       <c r="C63" s="25" t="n"/>
       <c r="D63" s="26" t="n"/>
       <c r="F63" s="179" t="n"/>
@@ -6648,7 +7200,10 @@
       <c r="M63" s="149" t="n"/>
     </row>
     <row r="64" ht="76.5" customHeight="1">
-      <c r="B64" s="24" t="n"/>
+      <c r="B64" s="24">
+        <f>B63+1</f>
+        <v/>
+      </c>
       <c r="C64" s="25" t="n"/>
       <c r="D64" s="26" t="n"/>
       <c r="F64" s="168" t="n"/>
@@ -6661,29 +7216,59 @@
       <c r="M64" s="153" t="n"/>
     </row>
     <row r="65" ht="76.5" customHeight="1">
-      <c r="B65" s="24" t="n"/>
+      <c r="B65" s="24">
+        <f>B64+1</f>
+        <v/>
+      </c>
       <c r="C65" s="25" t="n"/>
       <c r="D65" s="26" t="n"/>
     </row>
     <row r="66" ht="76.5" customHeight="1">
-      <c r="B66" s="24" t="n"/>
+      <c r="B66" s="24">
+        <f>B65+1</f>
+        <v/>
+      </c>
       <c r="C66" s="25" t="n"/>
       <c r="D66" s="26" t="n"/>
     </row>
     <row r="67" ht="76.5" customHeight="1">
-      <c r="B67" s="27" t="n"/>
+      <c r="B67" s="27">
+        <f>B66+1</f>
+        <v/>
+      </c>
       <c r="C67" s="28" t="n"/>
       <c r="D67" s="29" t="n"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="C68" s="15" t="n"/>
-      <c r="D68" s="16" t="n"/>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
+        </is>
+      </c>
+      <c r="D68" s="16">
+        <f>SUM(D63:D67)</f>
+        <v/>
+      </c>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="C69" s="15" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="K69" s="17" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Ημέρες Εργασίας Εβδομάδας:</t>
+        </is>
+      </c>
+      <c r="D69" s="16">
+        <f>COUNTA(D63:D67)</f>
+        <v/>
+      </c>
+      <c r="K69" s="17" t="inlineStr">
+        <is>
+          <t>Σύνολο Εργάσιμων Ημερών:</t>
+        </is>
+      </c>
+      <c r="L69" s="18">
+        <f>D69+L55</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="16.5" customHeight="1">
       <c r="B73" s="181" t="inlineStr">
@@ -6799,7 +7384,7 @@
         </is>
       </c>
       <c r="D3" s="185" t="n">
-        <v>46202</v>
+        <v>46237</v>
       </c>
       <c r="E3" s="163">
         <f>WEEKDAY(D3)</f>
@@ -6959,7 +7544,7 @@
         </is>
       </c>
       <c r="L13" s="18">
-        <f>D13+'4ος'!L55</f>
+        <f>D13+'4ος'!L69</f>
         <v/>
       </c>
     </row>
@@ -7714,72 +8299,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
-      <c r="B1" s="74" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
-        </is>
-      </c>
+      <c r="B1" s="74" t="n"/>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΑ</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>από Δευτέρα:</t>
-        </is>
-      </c>
-      <c r="D3" s="185" t="n">
-        <v>46237</v>
-      </c>
-      <c r="E3" s="163">
-        <f>WEEKDAY(D3)</f>
-        <v/>
-      </c>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="30" t="n"/>
+      <c r="E3" s="163" t="n"/>
     </row>
     <row r="4" ht="18.75" customHeight="1">
-      <c r="B4" s="34">
-        <f>('6ος'!D3-'Στοιχεία Πρακτικής'!C21)/7 + 1</f>
-        <v/>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>έως Παρασκευή:</t>
-        </is>
-      </c>
-      <c r="D4" s="31">
-        <f>D3+4</f>
-        <v/>
-      </c>
-      <c r="E4" s="163">
-        <f>WEEKDAY(D4)</f>
-        <v/>
-      </c>
+      <c r="B4" s="34" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="31" t="n"/>
+      <c r="E4" s="163" t="n"/>
     </row>
     <row r="6" ht="31.5" customHeight="1">
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>ΗΜΕΡΑ</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
- ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>ΩΡΕΣ</t>
-        </is>
-      </c>
-      <c r="F6" s="77" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="F6" s="77" t="n"/>
       <c r="G6" s="164" t="n"/>
       <c r="H6" s="164" t="n"/>
       <c r="I6" s="164" t="n"/>
@@ -7789,10 +8327,7 @@
       <c r="M6" s="165" t="n"/>
     </row>
     <row r="7" ht="76.5" customHeight="1">
-      <c r="B7" s="24">
-        <f>D3</f>
-        <v/>
-      </c>
+      <c r="B7" s="24" t="n"/>
       <c r="C7" s="22" t="n"/>
       <c r="D7" s="26" t="n"/>
       <c r="F7" s="166" t="n"/>
@@ -7805,10 +8340,7 @@
       <c r="M7" s="149" t="n"/>
     </row>
     <row r="8" ht="76.5" customHeight="1">
-      <c r="B8" s="24">
-        <f>B7+1</f>
-        <v/>
-      </c>
+      <c r="B8" s="24" t="n"/>
       <c r="C8" s="22" t="n"/>
       <c r="D8" s="26" t="n"/>
       <c r="F8" s="168" t="n"/>
@@ -7821,16 +8353,10 @@
       <c r="M8" s="153" t="n"/>
     </row>
     <row r="9" ht="76.5" customHeight="1">
-      <c r="B9" s="24">
-        <f>B8+1</f>
-        <v/>
-      </c>
+      <c r="B9" s="24" t="n"/>
       <c r="C9" s="22" t="n"/>
       <c r="D9" s="26" t="n"/>
-      <c r="F9" s="180">
-        <f>'1ος'!F9:M11</f>
-        <v/>
-      </c>
+      <c r="F9" s="180" t="n"/>
       <c r="G9" s="171" t="n"/>
       <c r="H9" s="171" t="n"/>
       <c r="I9" s="171" t="n"/>
@@ -7840,20 +8366,14 @@
       <c r="M9" s="172" t="n"/>
     </row>
     <row r="10" ht="76.5" customHeight="1">
-      <c r="B10" s="24">
-        <f>B9+1</f>
-        <v/>
-      </c>
+      <c r="B10" s="24" t="n"/>
       <c r="C10" s="22" t="n"/>
       <c r="D10" s="26" t="n"/>
       <c r="F10" s="173" t="n"/>
       <c r="M10" s="174" t="n"/>
     </row>
     <row r="11" ht="76.5" customHeight="1">
-      <c r="B11" s="27">
-        <f>B10+1</f>
-        <v/>
-      </c>
+      <c r="B11" s="27" t="n"/>
       <c r="C11" s="23" t="n"/>
       <c r="D11" s="29" t="n"/>
       <c r="F11" s="175" t="n"/>
@@ -7866,107 +8386,38 @@
       <c r="M11" s="177" t="n"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
-        </is>
-      </c>
-      <c r="D12" s="16">
-        <f>SUM(D7:D11)</f>
-        <v/>
-      </c>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="16" t="n"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="C13" s="15" t="inlineStr">
-        <is>
-          <t>Ημέρες Εργασίας Εβδομάδας:</t>
-        </is>
-      </c>
-      <c r="D13" s="16">
-        <f>COUNTA(D7:D11)</f>
-        <v/>
-      </c>
-      <c r="K13" s="17" t="inlineStr">
-        <is>
-          <t>Σύνολο Εργάσιμων Ημερών:</t>
-        </is>
-      </c>
-      <c r="L13" s="18">
-        <f>D13+'5ος'!L69</f>
-        <v/>
-      </c>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="K13" s="17" t="n"/>
+      <c r="L13" s="18" t="n"/>
     </row>
     <row r="14">
       <c r="N14" s="1" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="74" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
-        </is>
-      </c>
+      <c r="B15" s="74" t="n"/>
     </row>
     <row r="17" ht="18.75" customHeight="1">
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΑ</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>από Δευτέρα:</t>
-        </is>
-      </c>
-      <c r="D17" s="32">
-        <f>D3+7</f>
-        <v/>
-      </c>
-      <c r="E17" s="178">
-        <f>D17</f>
-        <v/>
-      </c>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="32" t="n"/>
+      <c r="E17" s="178" t="n"/>
     </row>
     <row r="18" ht="18.75" customHeight="1">
-      <c r="B18" s="12">
-        <f>B4+1</f>
-        <v/>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>έως Παρασκευή:</t>
-        </is>
-      </c>
-      <c r="D18" s="31">
-        <f>D17+4</f>
-        <v/>
-      </c>
-      <c r="E18" s="178">
-        <f>D18</f>
-        <v/>
-      </c>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="178" t="n"/>
     </row>
     <row r="20" ht="31.5" customHeight="1">
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>ΗΜΕΡΑ</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
- ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>ΩΡΕΣ</t>
-        </is>
-      </c>
-      <c r="F20" s="77" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="F20" s="77" t="n"/>
       <c r="G20" s="164" t="n"/>
       <c r="H20" s="164" t="n"/>
       <c r="I20" s="164" t="n"/>
@@ -7976,10 +8427,7 @@
       <c r="M20" s="165" t="n"/>
     </row>
     <row r="21" ht="76.5" customHeight="1">
-      <c r="B21" s="24">
-        <f>D17</f>
-        <v/>
-      </c>
+      <c r="B21" s="24" t="n"/>
       <c r="C21" s="22" t="n"/>
       <c r="D21" s="26" t="n"/>
       <c r="F21" s="179" t="n"/>
@@ -7992,10 +8440,7 @@
       <c r="M21" s="149" t="n"/>
     </row>
     <row r="22" ht="76.5" customHeight="1">
-      <c r="B22" s="24">
-        <f>B21+1</f>
-        <v/>
-      </c>
+      <c r="B22" s="24" t="n"/>
       <c r="C22" s="22" t="n"/>
       <c r="D22" s="26" t="n"/>
       <c r="F22" s="168" t="n"/>
@@ -8008,128 +8453,50 @@
       <c r="M22" s="153" t="n"/>
     </row>
     <row r="23" ht="76.5" customHeight="1">
-      <c r="B23" s="24">
-        <f>B22+1</f>
-        <v/>
-      </c>
+      <c r="B23" s="24" t="n"/>
       <c r="C23" s="22" t="n"/>
       <c r="D23" s="26" t="n"/>
     </row>
     <row r="24" ht="76.5" customHeight="1">
-      <c r="B24" s="24">
-        <f>B23+1</f>
-        <v/>
-      </c>
+      <c r="B24" s="24" t="n"/>
       <c r="C24" s="22" t="n"/>
       <c r="D24" s="26" t="n"/>
     </row>
     <row r="25" ht="76.5" customHeight="1">
-      <c r="B25" s="27">
-        <f>B24+1</f>
-        <v/>
-      </c>
+      <c r="B25" s="27" t="n"/>
       <c r="C25" s="23" t="n"/>
       <c r="D25" s="29" t="n"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
-        </is>
-      </c>
-      <c r="D26" s="16">
-        <f>SUM(D21:D25)</f>
-        <v/>
-      </c>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="16" t="n"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Ημέρες Εργασίας Εβδομάδας:</t>
-        </is>
-      </c>
-      <c r="D27" s="16">
-        <f>COUNTA(D21:D25)</f>
-        <v/>
-      </c>
-      <c r="K27" s="17" t="inlineStr">
-        <is>
-          <t>Σύνολο Εργάσιμων Ημερών:</t>
-        </is>
-      </c>
-      <c r="L27" s="18">
-        <f>D27+L13</f>
-        <v/>
-      </c>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="K27" s="17" t="n"/>
+      <c r="L27" s="18" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="74" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
-        </is>
-      </c>
+      <c r="B29" s="74" t="n"/>
     </row>
     <row r="31" ht="18.75" customHeight="1">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΑ</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>από Δευτέρα:</t>
-        </is>
-      </c>
-      <c r="D31" s="32">
-        <f>D17+7</f>
-        <v/>
-      </c>
-      <c r="E31" s="178">
-        <f>D31</f>
-        <v/>
-      </c>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="178" t="n"/>
     </row>
     <row r="32" ht="18.75" customHeight="1">
-      <c r="B32" s="12">
-        <f>B18+1</f>
-        <v/>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>έως Παρασκευή:</t>
-        </is>
-      </c>
-      <c r="D32" s="31">
-        <f>D31+4</f>
-        <v/>
-      </c>
-      <c r="E32" s="178">
-        <f>D32</f>
-        <v/>
-      </c>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="178" t="n"/>
     </row>
     <row r="34" ht="31.5" customHeight="1">
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>ΗΜΕΡΑ</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr">
-        <is>
-          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
- ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>ΩΡΕΣ</t>
-        </is>
-      </c>
-      <c r="F34" s="77" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="F34" s="77" t="n"/>
       <c r="G34" s="164" t="n"/>
       <c r="H34" s="164" t="n"/>
       <c r="I34" s="164" t="n"/>
@@ -8139,10 +8506,7 @@
       <c r="M34" s="165" t="n"/>
     </row>
     <row r="35" ht="76.5" customHeight="1">
-      <c r="B35" s="24">
-        <f>D31</f>
-        <v/>
-      </c>
+      <c r="B35" s="24" t="n"/>
       <c r="C35" s="25" t="n"/>
       <c r="D35" s="26" t="n"/>
       <c r="F35" s="179" t="n"/>
@@ -8155,10 +8519,7 @@
       <c r="M35" s="149" t="n"/>
     </row>
     <row r="36" ht="76.5" customHeight="1">
-      <c r="B36" s="24">
-        <f>B35+1</f>
-        <v/>
-      </c>
+      <c r="B36" s="24" t="n"/>
       <c r="C36" s="25" t="n"/>
       <c r="D36" s="26" t="n"/>
       <c r="F36" s="168" t="n"/>
@@ -8171,128 +8532,50 @@
       <c r="M36" s="153" t="n"/>
     </row>
     <row r="37" ht="76.5" customHeight="1">
-      <c r="B37" s="24">
-        <f>B36+1</f>
-        <v/>
-      </c>
+      <c r="B37" s="24" t="n"/>
       <c r="C37" s="25" t="n"/>
       <c r="D37" s="26" t="n"/>
     </row>
     <row r="38" ht="76.5" customHeight="1">
-      <c r="B38" s="24">
-        <f>B37+1</f>
-        <v/>
-      </c>
+      <c r="B38" s="24" t="n"/>
       <c r="C38" s="25" t="n"/>
       <c r="D38" s="26" t="n"/>
     </row>
     <row r="39" ht="76.5" customHeight="1">
-      <c r="B39" s="27">
-        <f>B38+1</f>
-        <v/>
-      </c>
+      <c r="B39" s="27" t="n"/>
       <c r="C39" s="28" t="n"/>
       <c r="D39" s="29" t="n"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
-        </is>
-      </c>
-      <c r="D40" s="16">
-        <f>SUM(D35:D39)</f>
-        <v/>
-      </c>
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="16" t="n"/>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>Ημέρες Εργασίας Εβδομάδας:</t>
-        </is>
-      </c>
-      <c r="D41" s="16">
-        <f>COUNTA(D35:D39)</f>
-        <v/>
-      </c>
-      <c r="K41" s="17" t="inlineStr">
-        <is>
-          <t>Σύνολο Εργάσιμων Ημερών:</t>
-        </is>
-      </c>
-      <c r="L41" s="18">
-        <f>D41+L27</f>
-        <v/>
-      </c>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="16" t="n"/>
+      <c r="K41" s="17" t="n"/>
+      <c r="L41" s="18" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="B43" s="74" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
-        </is>
-      </c>
+      <c r="B43" s="74" t="n"/>
     </row>
     <row r="45" ht="18.75" customHeight="1">
-      <c r="B45" s="10" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΑ</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>από Δευτέρα:</t>
-        </is>
-      </c>
-      <c r="D45" s="32">
-        <f>D31+7</f>
-        <v/>
-      </c>
-      <c r="E45" s="178">
-        <f>D45</f>
-        <v/>
-      </c>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="11" t="n"/>
+      <c r="D45" s="32" t="n"/>
+      <c r="E45" s="178" t="n"/>
     </row>
     <row r="46" ht="18.75" customHeight="1">
-      <c r="B46" s="12">
-        <f>B32+1</f>
-        <v/>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>έως Παρασκευή:</t>
-        </is>
-      </c>
-      <c r="D46" s="31">
-        <f>D45+4</f>
-        <v/>
-      </c>
-      <c r="E46" s="178">
-        <f>D46</f>
-        <v/>
-      </c>
+      <c r="B46" s="12" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="31" t="n"/>
+      <c r="E46" s="178" t="n"/>
     </row>
     <row r="48" ht="31.5" customHeight="1">
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>ΗΜΕΡΑ</t>
-        </is>
-      </c>
-      <c r="C48" s="14" t="inlineStr">
-        <is>
-          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
- ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>ΩΡΕΣ</t>
-        </is>
-      </c>
-      <c r="F48" s="77" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B48" s="13" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="13" t="n"/>
+      <c r="F48" s="77" t="n"/>
       <c r="G48" s="164" t="n"/>
       <c r="H48" s="164" t="n"/>
       <c r="I48" s="164" t="n"/>
@@ -8302,10 +8585,7 @@
       <c r="M48" s="165" t="n"/>
     </row>
     <row r="49" ht="76.5" customHeight="1">
-      <c r="B49" s="24">
-        <f>D45</f>
-        <v/>
-      </c>
+      <c r="B49" s="24" t="n"/>
       <c r="C49" s="25" t="n"/>
       <c r="D49" s="26" t="n"/>
       <c r="F49" s="179" t="n"/>
@@ -8318,10 +8598,7 @@
       <c r="M49" s="149" t="n"/>
     </row>
     <row r="50" ht="76.5" customHeight="1">
-      <c r="B50" s="24">
-        <f>B49+1</f>
-        <v/>
-      </c>
+      <c r="B50" s="24" t="n"/>
       <c r="C50" s="25" t="n"/>
       <c r="D50" s="26" t="n"/>
       <c r="F50" s="168" t="n"/>
@@ -8334,128 +8611,50 @@
       <c r="M50" s="153" t="n"/>
     </row>
     <row r="51" ht="76.5" customHeight="1">
-      <c r="B51" s="24">
-        <f>B50+1</f>
-        <v/>
-      </c>
+      <c r="B51" s="24" t="n"/>
       <c r="C51" s="25" t="n"/>
       <c r="D51" s="26" t="n"/>
     </row>
     <row r="52" ht="76.5" customHeight="1">
-      <c r="B52" s="24">
-        <f>B51+1</f>
-        <v/>
-      </c>
+      <c r="B52" s="24" t="n"/>
       <c r="C52" s="25" t="n"/>
       <c r="D52" s="26" t="n"/>
     </row>
     <row r="53" ht="76.5" customHeight="1">
-      <c r="B53" s="27">
-        <f>B52+1</f>
-        <v/>
-      </c>
+      <c r="B53" s="27" t="n"/>
       <c r="C53" s="28" t="n"/>
       <c r="D53" s="29" t="n"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
-        </is>
-      </c>
-      <c r="D54" s="16">
-        <f>SUM(D49:D53)</f>
-        <v/>
-      </c>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="16" t="n"/>
     </row>
     <row r="55" ht="19.5" customHeight="1">
-      <c r="C55" s="15" t="inlineStr">
-        <is>
-          <t>Ημέρες Εργασίας Εβδομάδας:</t>
-        </is>
-      </c>
-      <c r="D55" s="16">
-        <f>COUNTA(D49:D53)</f>
-        <v/>
-      </c>
-      <c r="K55" s="17" t="inlineStr">
-        <is>
-          <t>Σύνολο Εργάσιμων Ημερών:</t>
-        </is>
-      </c>
-      <c r="L55" s="18">
-        <f>D55+L41</f>
-        <v/>
-      </c>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="16" t="n"/>
+      <c r="K55" s="17" t="n"/>
+      <c r="L55" s="18" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="74" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΟ ΦΥΛΛΟ ΠΡΑΚΤΙΚΗΣ ΑΣΚΗΣΗΣ</t>
-        </is>
-      </c>
+      <c r="B57" s="74" t="n"/>
     </row>
     <row r="59" ht="18.75" customHeight="1">
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΑ</t>
-        </is>
-      </c>
-      <c r="C59" s="11" t="inlineStr">
-        <is>
-          <t>από Δευτέρα:</t>
-        </is>
-      </c>
-      <c r="D59" s="32">
-        <f>D45+7</f>
-        <v/>
-      </c>
-      <c r="E59" s="178">
-        <f>D59</f>
-        <v/>
-      </c>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="32" t="n"/>
+      <c r="E59" s="178" t="n"/>
     </row>
     <row r="60" ht="18.75" customHeight="1">
-      <c r="B60" s="12">
-        <f>B46+1</f>
-        <v/>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>έως Παρασκευή:</t>
-        </is>
-      </c>
-      <c r="D60" s="31">
-        <f>D59+4</f>
-        <v/>
-      </c>
-      <c r="E60" s="178">
-        <f>D60</f>
-        <v/>
-      </c>
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="11" t="n"/>
+      <c r="D60" s="31" t="n"/>
+      <c r="E60" s="178" t="n"/>
     </row>
     <row r="62" ht="31.5" customHeight="1">
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>ΗΜΕΡΑ</t>
-        </is>
-      </c>
-      <c r="C62" s="14" t="inlineStr">
-        <is>
-          <t>ΠΕΡΙΛΗΨΗ ΕΡΓΑΣΙΩΝ
- ΠΟΥ ΕΚΕΤΕΛΕΣΤΗΚΑΝ</t>
-        </is>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
-        <is>
-          <t>ΩΡΕΣ</t>
-        </is>
-      </c>
-      <c r="F62" s="77" t="inlineStr">
-        <is>
-          <t>ΕΒΔΟΜΑΔΙΑΙΕΣ ΣΗΜΕΙΩΣΕΙΣ - ΠΑΡΑΤΗΡΗΣΕΙΣ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B62" s="13" t="n"/>
+      <c r="C62" s="14" t="n"/>
+      <c r="D62" s="13" t="n"/>
+      <c r="F62" s="77" t="n"/>
       <c r="G62" s="164" t="n"/>
       <c r="H62" s="164" t="n"/>
       <c r="I62" s="164" t="n"/>
@@ -8465,10 +8664,7 @@
       <c r="M62" s="165" t="n"/>
     </row>
     <row r="63" ht="76.5" customHeight="1">
-      <c r="B63" s="24">
-        <f>D59</f>
-        <v/>
-      </c>
+      <c r="B63" s="24" t="n"/>
       <c r="C63" s="25" t="n"/>
       <c r="D63" s="26" t="n"/>
       <c r="F63" s="179" t="n"/>
@@ -8481,10 +8677,7 @@
       <c r="M63" s="149" t="n"/>
     </row>
     <row r="64" ht="76.5" customHeight="1">
-      <c r="B64" s="24">
-        <f>B63+1</f>
-        <v/>
-      </c>
+      <c r="B64" s="24" t="n"/>
       <c r="C64" s="25" t="n"/>
       <c r="D64" s="26" t="n"/>
       <c r="F64" s="168" t="n"/>
@@ -8497,66 +8690,32 @@
       <c r="M64" s="153" t="n"/>
     </row>
     <row r="65" ht="76.5" customHeight="1">
-      <c r="B65" s="24">
-        <f>B64+1</f>
-        <v/>
-      </c>
+      <c r="B65" s="24" t="n"/>
       <c r="C65" s="25" t="n"/>
       <c r="D65" s="26" t="n"/>
     </row>
     <row r="66" ht="76.5" customHeight="1">
-      <c r="B66" s="24">
-        <f>B65+1</f>
-        <v/>
-      </c>
+      <c r="B66" s="24" t="n"/>
       <c r="C66" s="25" t="n"/>
       <c r="D66" s="26" t="n"/>
     </row>
     <row r="67" ht="76.5" customHeight="1">
-      <c r="B67" s="27">
-        <f>B66+1</f>
-        <v/>
-      </c>
+      <c r="B67" s="27" t="n"/>
       <c r="C67" s="28" t="n"/>
       <c r="D67" s="29" t="n"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="C68" s="15" t="inlineStr">
-        <is>
-          <t>Σύνολο Εβδομαδιαίων Ωρών:</t>
-        </is>
-      </c>
-      <c r="D68" s="16">
-        <f>SUM(D63:D67)</f>
-        <v/>
-      </c>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="16" t="n"/>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>Ημέρες Εργασίας Εβδομάδας:</t>
-        </is>
-      </c>
-      <c r="D69" s="16">
-        <f>COUNTA(D63:D67)</f>
-        <v/>
-      </c>
-      <c r="K69" s="17" t="inlineStr">
-        <is>
-          <t>Σύνολο Εργάσιμων Ημερών:</t>
-        </is>
-      </c>
-      <c r="L69" s="18">
-        <f>D69+L55</f>
-        <v/>
-      </c>
+      <c r="C69" s="15" t="n"/>
+      <c r="D69" s="16" t="n"/>
+      <c r="K69" s="17" t="n"/>
+      <c r="L69" s="18" t="n"/>
     </row>
     <row r="73" ht="16.5" customHeight="1">
-      <c r="B73" s="181" t="inlineStr">
-        <is>
-          <t>ΜΗΝΙΑΙΑ ΕΚΘΕΣΗ ΕΡΓΑΣΙΑΚΩΝ ΕΜΠΕΙΡΙΩΝ ΑΣΚΟΥΜΕΝΟΥ</t>
-        </is>
-      </c>
+      <c r="B73" s="181" t="n"/>
       <c r="C73" s="164" t="n"/>
       <c r="D73" s="165" t="n"/>
     </row>
@@ -8566,11 +8725,7 @@
       <c r="D74" s="183" t="n"/>
     </row>
     <row r="77" ht="16.5" customHeight="1">
-      <c r="B77" s="181" t="inlineStr">
-        <is>
-          <t>ΜΗΝΙΑΙΑ ΕΚΘΕΣΗ ΕΠΟΠΤΗ ΕΚΠΑΙΔΕΥΤΙΚΟΥ</t>
-        </is>
-      </c>
+      <c r="B77" s="181" t="n"/>
       <c r="C77" s="164" t="n"/>
       <c r="D77" s="165" t="n"/>
     </row>
@@ -8823,7 +8978,7 @@
         </is>
       </c>
       <c r="L13" s="18">
-        <f>D13+'6ος'!L69</f>
+        <f>D13+'5ος'!L69</f>
         <v/>
       </c>
     </row>

</xml_diff>